<commit_message>
[control] Point the elevator and rudder at the tail arm that was decided
Both sheets held their own typed number for the same length: the elevator
put the tail station 5.100 m behind the wing AC, the rudder gave the fin
an arm of 4.299 m, and Cruise carried 16.728 ft. None was derived and no
two agreed. Control 01 exists to settle it, so they now read it.

The elevator's tail station becomes the wing station plus the carried
arm, and the rudder's fin arm is the carried arm - which is also the
length its volume coefficient is defined on, though the field had been
labelled from the centre of gravity. Both move from the entry sections to
CARRIED · UPSTREAM.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VwapbkU1h5f4XmJdApLQP1
</commit_message>
<xml_diff>
--- a/spreadsheets/3.Control Surface Sizing.xlsx
+++ b/spreadsheets/3.Control Surface Sizing.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Geoffrey Nyaga\Desktop\Spreadsheets backup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geoff/Documents/code/Kenya-One-Project/spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01006089-97CF-4344-8CEE-8EE1F39E3684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="36080" windowHeight="20920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aileron" sheetId="1" r:id="rId1"/>
@@ -20,22 +21,33 @@
     <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
   </externalReferences>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="G24" authorId="0" shapeId="0">
+    <comment ref="G24" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -65,13 +77,13 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Geoffrey Nyaga</author>
     <author>Windows User</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -95,7 +107,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B2" authorId="1" shapeId="0">
+    <comment ref="B2" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
       <text>
         <r>
           <rPr>
@@ -120,13 +132,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="A3" authorId="0" shapeId="0">
+    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -135,22 +147,31 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-fuselage diameter</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fuselage diameter</t>
         </r>
       </text>
     </comment>
-    <comment ref="A4" authorId="0" shapeId="0">
+    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -159,16 +180,25 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-fuselage length</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>fuselage length</t>
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="1" shapeId="0">
+    <comment ref="A13" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
       <text>
         <r>
           <rPr>
@@ -193,7 +223,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A31" authorId="1" shapeId="0">
+    <comment ref="A31" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
       <text>
         <r>
           <rPr>
@@ -218,7 +248,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J31" authorId="1" shapeId="0">
+    <comment ref="J31" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0100-000007000000}">
       <text>
         <r>
           <rPr>
@@ -247,13 +277,13 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Windows User</author>
     <author>Geoffrey Nyaga</author>
   </authors>
   <commentList>
-    <comment ref="D2" authorId="0" shapeId="0">
+    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
           <rPr>
@@ -277,7 +307,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G2" authorId="1" shapeId="0">
+    <comment ref="G2" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
       <text>
         <r>
           <rPr>
@@ -301,7 +331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D3" authorId="0" shapeId="0">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000003000000}">
       <text>
         <r>
           <rPr>
@@ -325,7 +355,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E3" authorId="0" shapeId="0">
+    <comment ref="E3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000004000000}">
       <text>
         <r>
           <rPr>
@@ -350,7 +380,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="0" shapeId="0">
+    <comment ref="A14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000005000000}">
       <text>
         <r>
           <rPr>
@@ -375,7 +405,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B33" authorId="0" shapeId="0">
+    <comment ref="B33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000006000000}">
       <text>
         <r>
           <rPr>
@@ -3254,8 +3284,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="24" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3426,6 +3456,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -3517,7 +3560,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3538,7 +3581,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3548,7 +3590,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
@@ -3563,9 +3604,6 @@
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3810,7 +3848,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -3854,7 +3892,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3988,6 +4025,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-74FE-6A47-B5FC-1F99B152DCEB}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -4047,6 +4089,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-74FE-6A47-B5FC-1F99B152DCEB}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -4106,6 +4153,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-74FE-6A47-B5FC-1F99B152DCEB}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -4430,7 +4482,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -4601,33 +4653,38 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>-17.481001755809022</c:v>
+                  <c:v>-18.168554337563641</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-15.15316089761907</c:v>
+                  <c:v>-15.840713479373687</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-12.785660214312358</c:v>
+                  <c:v>-13.473212796066976</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-9.3125038299474845</c:v>
+                  <c:v>-10.000056411702106</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-5.2280719219343936</c:v>
+                  <c:v>-5.9156245036890125</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-3.0093681694334524</c:v>
+                  <c:v>-3.6969207511880722</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-1.6715597843447585</c:v>
+                  <c:v>-2.3591123660993776</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-0.47938984202989654</c:v>
+                  <c:v>-1.1669424237845154</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C09D-CE4B-98C1-5F3BDEB17DAD}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -4699,33 +4756,38 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>-19.569066200539144</c:v>
+                  <c:v>-20.352017865551858</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-16.889135801130667</c:v>
+                  <c:v>-17.672087466143378</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-14.163546966528189</c:v>
+                  <c:v>-14.946498631540898</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-10.165070290765875</c:v>
+                  <c:v>-10.948021955778588</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-5.4628617200693981</c:v>
+                  <c:v>-6.2458133850821085</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-2.9085755829009377</c:v>
+                  <c:v>-3.6915272479136494</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-1.3684216040887851</c:v>
+                  <c:v>-2.1513732691014962</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.0658915362010179E-3</c:v>
+                  <c:v>-0.77888577347650978</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C09D-CE4B-98C1-5F3BDEB17DAD}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -5101,7 +5163,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -5307,33 +5369,38 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>-24.400307338363746</c:v>
+                  <c:v>-25.087859920118362</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-21.2470629266572</c:v>
+                  <c:v>-21.934615508411817</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-18.040096147513609</c:v>
+                  <c:v>-18.727648729268225</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-13.335431341304691</c:v>
+                  <c:v>-14.022983923059309</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-7.8027455292030039</c:v>
+                  <c:v>-8.4902981109576228</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-4.7973359522588774</c:v>
+                  <c:v>-5.4848885340134963</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-2.9851687676450704</c:v>
+                  <c:v>-3.6727213493996893</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1.3702803635761287</c:v>
+                  <c:v>-2.0578329453307478</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F162-E74B-8F9B-887BFA47B9C0}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -5405,33 +5472,38 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>-27.534927487080761</c:v>
+                  <c:v>-28.317879152093475</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-23.904749966153471</c:v>
+                  <c:v>-24.687701631166185</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-20.212724486369282</c:v>
+                  <c:v>-20.995676151381996</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-14.796471829394218</c:v>
+                  <c:v>-15.579423494406925</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-8.4269587047915326</c:v>
+                  <c:v>-9.2099103698042448</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-4.9669762667357551</c:v>
+                  <c:v>-5.7499279317484655</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-2.8807159840490586</c:v>
+                  <c:v>-3.6636676490617694</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1.0215732035233613</c:v>
+                  <c:v>-1.8045248685360724</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F162-E74B-8F9B-887BFA47B9C0}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -7529,7 +7601,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="3" name="TextBox 2"/>
+            <xdr:cNvPr id="3" name="TextBox 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -7565,10 +7643,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -7645,7 +7720,13 @@
     <xdr:ext cx="65" cy="172227"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="TextBox 3"/>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -7699,7 +7780,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="6" name="Straight Arrow Connector 5"/>
+        <xdr:cNvPr id="6" name="Straight Arrow Connector 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -7746,7 +7833,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="8" name="Straight Arrow Connector 7"/>
+        <xdr:cNvPr id="8" name="Straight Arrow Connector 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -7793,7 +7886,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="9" name="Chart 8"/>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -7823,7 +7922,13 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="TextBox 9"/>
+        <xdr:cNvPr id="10" name="TextBox 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -7905,7 +8010,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="3" name="Straight Arrow Connector 2"/>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -7952,7 +8063,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -7982,7 +8099,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="5" name="Straight Arrow Connector 4"/>
+        <xdr:cNvPr id="5" name="Straight Arrow Connector 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8029,7 +8152,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="7" name="Straight Arrow Connector 6"/>
+        <xdr:cNvPr id="7" name="Straight Arrow Connector 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8076,7 +8205,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -8111,7 +8246,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="3" name="Straight Arrow Connector 2"/>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8158,7 +8299,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="5" name="Straight Arrow Connector 4"/>
+        <xdr:cNvPr id="5" name="Straight Arrow Connector 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8205,7 +8352,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="4" name="Straight Arrow Connector 3"/>
+        <xdr:cNvPr id="4" name="Straight Arrow Connector 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8252,7 +8405,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="12" name="Straight Connector 11"/>
+        <xdr:cNvPr id="12" name="Straight Connector 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8296,7 +8455,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="18" name="Straight Arrow Connector 17"/>
+        <xdr:cNvPr id="18" name="Straight Arrow Connector 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000012000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8343,7 +8508,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="24" name="Straight Arrow Connector 23"/>
+        <xdr:cNvPr id="24" name="Straight Arrow Connector 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000018000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -8379,8 +8550,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Cost Analysis"/>
       <sheetName val="MTOW &amp; WEIGHTS"/>
@@ -8443,7 +8617,7 @@
         </row>
         <row r="14">
           <cell r="L14">
-            <v>0.39080126986823693</v>
+            <v>0.33033961893414038</v>
           </cell>
         </row>
         <row r="15">
@@ -8473,8 +8647,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="take-off"/>
       <sheetName val="climb"/>
@@ -8484,6 +8661,11 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0">
+        <row r="7">
+          <cell r="C7">
+            <v>520</v>
+          </cell>
+        </row>
         <row r="16">
           <cell r="B16">
             <v>140</v>
@@ -8495,8 +8677,20 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
+      <sheetData sheetId="1">
+        <row r="19">
+          <cell r="B19">
+            <v>75.225033459938444</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2">
+        <row r="7">
+          <cell r="B7">
+            <v>0.75</v>
+          </cell>
+        </row>
+      </sheetData>
       <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
     </sheetDataSet>
@@ -8505,59 +8699,59 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="H36:Z45" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="H36:Z45" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="19">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2">
       <calculatedColumnFormula>B$34</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" name="Column3">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3">
       <calculatedColumnFormula>0.5*1.225*(H36*0.514)^2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" name="Column4" headerRowDxfId="19">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4" headerRowDxfId="19">
       <calculatedColumnFormula>(2*Aileron!B$5*9.81)/(1.225*Aileron!B$7*(Elevator!H36*0.514)^2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" name="Column5" headerRowDxfId="18">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Column5" headerRowDxfId="18">
       <calculatedColumnFormula>-(( (B$13 *(B$22-B$23)/(J36*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!N36-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" name="Column6" dataDxfId="17">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Column6" dataDxfId="17">
       <calculatedColumnFormula>L36*57.3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Column7">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Column7">
       <calculatedColumnFormula>-(( (B$13 *(B$22-B$23)/(J36*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K36-Elevator!B$7)*R36)/ ((Aileron!B$11*Elevator!S36)-(R36*Elevator!B$33))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" name="Column8" dataDxfId="16">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Column8" dataDxfId="16">
       <calculatedColumnFormula>#REF!*57.3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" name="Column9">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Column9">
       <calculatedColumnFormula>5.2414</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" name="Column10">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Column10">
       <calculatedColumnFormula>P36*Aileron!B$8/(Aileron!B$7*Aileron!B$15)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" name="Column11">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Column11">
       <calculatedColumnFormula>Aileron!B$11*((T36)/Aileron!B$15)-(H$3*H$6*(Aileron!B$8/Aileron!B$7)*(B$24/Aileron!B$15)*(1-Elevator!H$24))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" name="Column12">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Column12">
       <calculatedColumnFormula>-H$3*H$6*Q36*B$40*B$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" name="Column13"/>
-    <tableColumn id="14" name="Column14" headerRowDxfId="15">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Column13"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Column14" headerRowDxfId="15">
       <calculatedColumnFormula>(2*Aileron!B$5*9.81)/(0.90434*Aileron!B$7*(Elevator!H36*0.514)^2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" name="Column15" headerRowDxfId="14">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Column15" headerRowDxfId="14">
       <calculatedColumnFormula>0.5*0.90434*(H36*0.514)^2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" name="Column16">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Column16">
       <calculatedColumnFormula>-(( (B$13 *(B$22-B$23)/(V36*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U36-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" name="Column17" dataDxfId="13">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Column17" dataDxfId="13">
       <calculatedColumnFormula>#REF!*57.3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" name="Column18">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Column18">
       <calculatedColumnFormula>-(( (B$13 *(B$22-B$23)/(V36*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(X36-Elevator!B$7)*R36)/ ((Aileron!B$11*Elevator!S36)-(R36*Elevator!B$33))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" name="Column19" dataDxfId="12">
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Column19" dataDxfId="12">
       <calculatedColumnFormula>Y36*57.3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8566,61 +8760,61 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="D2:E8" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table2" displayName="Table2" ref="D2:E8" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="11"/>
-    <tableColumn id="2" name="Column2" headerRowDxfId="10" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Column1" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Column2" headerRowDxfId="10" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:B15" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:B15" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" headerRowDxfId="8" dataDxfId="7"/>
-    <tableColumn id="2" name="Column2" headerRowDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Column1" headerRowDxfId="8" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Column2" headerRowDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="G2:H9" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="G2:H9" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="5"/>
-    <tableColumn id="2" name="Column2" headerRowDxfId="4" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Column1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Column2" headerRowDxfId="4" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="D15:E23" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table5" displayName="Table5" ref="D15:E23" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Column2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="A17:B24" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table6" displayName="Table6" ref="A17:B24" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="2"/>
-    <tableColumn id="2" name="Column2" headerRowDxfId="1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Column1" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Column2" headerRowDxfId="1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table7" displayName="Table7" ref="F29:H33" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Table7" displayName="Table7" ref="F29:H33" headerRowCount="0" totalsRowShown="0">
   <tableColumns count="3">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Column2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Column3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8888,30 +9082,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A5:M46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="10.28515625" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5">
         <f>[1]!Table9[[#Headers],[5850]]/2.204623</f>
         <v>2653.514909351848</v>
       </c>
       <c r="C5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
       <c r="G5" t="s">
         <v>12</v>
       </c>
@@ -8932,11 +9126,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6">
         <f>'[1]Sref and POWER SIZING'!$B$17</f>
         <v>7.8</v>
       </c>
@@ -8960,11 +9154,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7">
         <f>'[1]Sref and POWER SIZING'!$H$80</f>
         <v>23.951178858082848</v>
       </c>
@@ -8982,11 +9176,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <v>6.343</v>
       </c>
       <c r="C8" t="s">
@@ -9004,26 +9198,26 @@
       <c r="K8" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="10">
         <v>0.09</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <v>4.9875999999999996</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="16">
+      <c r="B10">
         <f>'[1]Sref and POWER SIZING'!$B$11</f>
         <v>61</v>
       </c>
@@ -9040,36 +9234,36 @@
       <c r="G10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="10">
         <v>0.41</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
     </row>
-    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11">
         <f>[1]!Table21[[#This Row],[Column4]]</f>
         <v>4.7321150412315607</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12">
         <f>'[1]Wing &amp; Airfoil'!$B$5</f>
         <v>0.45</v>
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>204</v>
       </c>
@@ -9088,7 +9282,7 @@
         <v>6.1506818326378951</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>203</v>
       </c>
@@ -9104,7 +9298,7 @@
         <v>4.1004545550919298</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>201</v>
       </c>
@@ -9123,7 +9317,7 @@
         <v>0.16719852854795431</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>170</v>
       </c>
@@ -9131,34 +9325,34 @@
         <f>B13^2*B5*0.34^2/(4*9.81)</f>
         <v>1460.4001339948557</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
       <c r="G16" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="11">
         <v>17</v>
       </c>
       <c r="I16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <v>3.8</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="12">
         <v>1.3</v>
       </c>
       <c r="C18" s="4" t="s">
@@ -9179,22 +9373,22 @@
         <v>4.9608784331752469E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <v>5</v>
       </c>
       <c r="C19" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="10">
         <v>0.8</v>
       </c>
       <c r="D20" s="4" t="s">
@@ -9224,7 +9418,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>28</v>
       </c>
@@ -9246,12 +9440,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="18" x14ac:dyDescent="0.35">
-      <c r="A22" s="32" t="s">
+    <row r="22" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="A22" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
       <c r="D22" t="s">
         <v>32</v>
       </c>
@@ -9260,7 +9454,7 @@
         <v>2.7336363700612867</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
         <v>30</v>
       </c>
@@ -9278,33 +9472,33 @@
       <c r="I23" t="s">
         <v>41</v>
       </c>
-      <c r="J23" s="15" t="s">
+      <c r="J23" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="G24" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="16">
+      <c r="H24">
         <v>1.8</v>
       </c>
       <c r="I24" t="s">
         <v>41</v>
       </c>
-      <c r="J24" s="21" t="s">
+      <c r="J24" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="14"/>
+      <c r="B25" s="13"/>
     </row>
-    <row r="26" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -9316,8 +9510,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="18" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:12" ht="17" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>44</v>
       </c>
       <c r="B27" s="8">
@@ -9328,7 +9522,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>45</v>
       </c>
@@ -9340,7 +9534,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -9349,7 +9543,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
@@ -9358,7 +9552,7 @@
       </c>
       <c r="D32" s="1"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>0</v>
       </c>
@@ -9367,7 +9561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>5</v>
       </c>
@@ -9376,7 +9570,7 @@
         <v>0.24773745808213105</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>10</v>
       </c>
@@ -9385,7 +9579,7 @@
         <v>0.35035367312758586</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>15</v>
       </c>
@@ -9394,7 +9588,7 @@
         <v>0.42909386433621594</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>20</v>
       </c>
@@ -9403,7 +9597,7 @@
         <v>0.49547491616426209</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>25</v>
       </c>
@@ -9412,7 +9606,7 @@
         <v>0.55395779684464963</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>30</v>
       </c>
@@ -9421,7 +9615,7 @@
         <v>0.60683036247535749</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>40</v>
       </c>
@@ -9430,7 +9624,7 @@
         <v>0.70070734625517173</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>60</v>
       </c>
@@ -9439,7 +9633,7 @@
         <v>0.85818772867243187</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" ht="17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>40</v>
       </c>
@@ -9447,7 +9641,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44">
         <f>H$23</f>
         <v>0.60680812221158964</v>
@@ -9462,7 +9656,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45">
         <f t="shared" ref="A45:A46" si="1">H$23</f>
         <v>0.60680812221158964</v>
@@ -9477,7 +9671,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46">
         <f t="shared" si="1"/>
         <v>0.60680812221158964</v>
@@ -9504,35 +9698,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:Z45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="11" customWidth="1"/>
     <col min="4" max="16" width="11" customWidth="1"/>
     <col min="17" max="26" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
+    <row r="1" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="11">
+      <c r="B1" s="10">
         <v>-21</v>
       </c>
       <c r="C1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="13" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="18.75" x14ac:dyDescent="0.35">
-      <c r="A2" s="31" t="s">
+    <row r="2" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
         <v>215</v>
       </c>
       <c r="B2">
@@ -9542,43 +9736,43 @@
       <c r="C2" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="10">
         <v>0.8</v>
       </c>
-      <c r="G2" s="31" t="s">
+      <c r="G2" s="28" t="s">
         <v>226</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="10">
         <v>0.10100000000000001</v>
       </c>
       <c r="I2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="31" t="s">
+    <row r="3" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
         <v>216</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="10">
         <v>1.3462000000000001</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="D3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3">
         <f>'[1]Wing &amp; Airfoil'!$L$15</f>
         <v>-7.1677464485709705E-2</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="28" t="s">
         <v>227</v>
       </c>
-      <c r="H3" s="16">
+      <c r="H3">
         <f>(H2/(1+(H2/(3.142*Aileron!B17))))*57.3</f>
         <v>5.7387544707074394</v>
       </c>
@@ -9586,64 +9780,64 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A4" s="31" t="s">
+    <row r="4" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4" s="28" t="s">
         <v>217</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <v>9.1</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4">
         <f>'[1]Wing &amp; Airfoil'!$B$15</f>
         <v>1.8</v>
       </c>
       <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="31" t="s">
+      <c r="G4" s="28" t="s">
         <v>228</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>-0.35660999999999998</v>
       </c>
       <c r="I4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A5" s="31" t="s">
+    <row r="5" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5">
         <f>'[1]Sref and POWER SIZING'!$B$25</f>
         <v>3.0219944010805921E-2</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <f>'[1]Wing &amp; Airfoil'!$B$29</f>
         <v>0.247</v>
       </c>
-      <c r="G5" s="30" t="s">
+      <c r="G5" s="27" t="s">
         <v>229</v>
       </c>
-      <c r="H5" s="16">
+      <c r="H5">
         <f>Aileron!B20</f>
         <v>0.8</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="31" t="s">
+    <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6">
         <f>'[2]take-off'!$B$16</f>
         <v>140</v>
       </c>
@@ -9653,86 +9847,86 @@
       <c r="D6" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6">
         <f>'[1]Wing &amp; Airfoil'!$B$25</f>
         <v>14</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>0.98</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A7" s="31" t="s">
+    <row r="7" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
         <v>233</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7">
         <f>'[1]Wing &amp; Airfoil'!$L$14</f>
-        <v>0.39080126986823693</v>
+        <v>0.33033961893414038</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7">
         <f>'[2]take-off'!$M$17</f>
         <v>1.4869053204776603</v>
       </c>
-      <c r="G7" s="30" t="s">
+      <c r="G7" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <v>14</v>
       </c>
       <c r="I7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A8" s="31" t="s">
+    <row r="8" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A8" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <v>2.58E-2</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8">
         <f>E3</f>
         <v>-7.1677464485709705E-2</v>
       </c>
-      <c r="G8" s="30" t="s">
+      <c r="G8" s="27" t="s">
         <v>231</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <v>0</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="31" t="s">
+    <row r="9" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A9" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9">
         <f>'[1]Sref and POWER SIZING'!$B$18</f>
         <v>0.75552604922347777</v>
       </c>
-      <c r="G9" s="30" t="s">
+      <c r="G9" s="27" t="s">
         <v>232</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="10">
         <v>5.0999999999999996</v>
       </c>
       <c r="I9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="31" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="28" t="s">
         <v>69</v>
       </c>
       <c r="B10">
@@ -9754,11 +9948,11 @@
         <v>0.14962326466758191</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A11" s="30" t="s">
+    <row r="11" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A11" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11">
         <f>'[1]Sref and POWER SIZING'!$B$29</f>
         <v>9.014705184847549E-2</v>
       </c>
@@ -9773,8 +9967,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="18.75" x14ac:dyDescent="0.35">
-      <c r="A12" s="31" t="s">
+    <row r="12" spans="1:9" ht="18" x14ac:dyDescent="0.25">
+      <c r="A12" s="28" t="s">
         <v>65</v>
       </c>
       <c r="B12">
@@ -9784,7 +9978,7 @@
       <c r="D12" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="10">
         <v>9</v>
       </c>
       <c r="F12" t="s">
@@ -9801,19 +9995,19 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="31" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <v>3800</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="31" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="28" t="s">
         <v>72</v>
       </c>
       <c r="B14">
@@ -9824,8 +10018,8 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="18" x14ac:dyDescent="0.35">
-      <c r="A15" s="31" t="s">
+    <row r="15" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+      <c r="A15" s="28" t="s">
         <v>73</v>
       </c>
       <c r="B15">
@@ -9846,7 +10040,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="17" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>179</v>
       </c>
@@ -9860,15 +10054,15 @@
       <c r="G16" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="10">
         <v>0.477468</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A17" s="31" t="s">
+    <row r="17" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A17" s="28" t="s">
         <v>218</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <v>0</v>
       </c>
       <c r="D17" t="s">
@@ -9884,15 +10078,15 @@
       <c r="G17" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="10">
         <v>0.17684</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A18" s="31" t="s">
+    <row r="18" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
         <v>219</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="10">
         <v>-0.61894000000000005</v>
       </c>
       <c r="C18" t="s">
@@ -9909,11 +10103,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A19" s="31" t="s">
+    <row r="19" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A19" s="28" t="s">
         <v>220</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <v>1.6</v>
       </c>
       <c r="D19" t="s">
@@ -9927,11 +10121,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A20" s="31" t="s">
+    <row r="20" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A20" s="28" t="s">
         <v>221</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="10">
         <v>0</v>
       </c>
       <c r="D20" t="s">
@@ -9945,19 +10139,19 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A21" s="31" t="s">
+    <row r="21" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A21" s="28" t="s">
         <v>222</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <v>-0.477468</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A22" s="31" t="s">
+    <row r="22" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A22" s="28" t="s">
         <v>223</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="10">
         <v>1.5</v>
       </c>
       <c r="D22" t="s">
@@ -9981,11 +10175,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A23" s="31" t="s">
+    <row r="23" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A23" s="28" t="s">
         <v>224</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <v>1.3</v>
       </c>
       <c r="D23" t="s">
@@ -10006,11 +10200,11 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="A24" s="31" t="s">
+    <row r="24" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A24" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="10">
         <v>4.6225319999999996</v>
       </c>
       <c r="G24" s="1" t="s">
@@ -10024,7 +10218,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="G25" s="3" t="s">
         <v>76</v>
       </c>
@@ -10036,7 +10230,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>81</v>
       </c>
@@ -10055,7 +10249,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>82</v>
       </c>
@@ -10063,18 +10257,18 @@
         <f>((B26/57.3)+(E23/H3))/(B1/57.3)</f>
         <v>0.49732426951731462</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
     </row>
-    <row r="29" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>83</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="10">
         <v>0.35</v>
       </c>
       <c r="F29" t="s">
@@ -10098,7 +10292,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>85</v>
       </c>
@@ -10126,14 +10320,14 @@
       <c r="K30" t="s">
         <v>24</v>
       </c>
-      <c r="L30" s="22" t="s">
+      <c r="L30" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="M30" s="19"/>
-      <c r="N30" s="19"/>
-      <c r="O30" s="19"/>
+      <c r="M30" s="17"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="17"/>
     </row>
-    <row r="31" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>134</v>
       </c>
@@ -10159,7 +10353,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>135</v>
       </c>
@@ -10175,13 +10369,13 @@
       </c>
       <c r="G32">
         <f>-(( ( B13*(B22-B23)/(G30*Aileron!B7*Aileron!B15)+Elevator!E8))*Aileron!B11 +(Elevator!G31-Elevator!B7)*Elevator!G29)/ ((Aileron!B11*Elevator!B32)-(Elevator!G29*Elevator!B33))</f>
-        <v>-2.9172073025213938E-2</v>
+        <v>-4.117124548166453E-2</v>
       </c>
       <c r="H32" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="33" spans="1:26" ht="18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:26" ht="17" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>136</v>
       </c>
@@ -10194,13 +10388,13 @@
       </c>
       <c r="G33" s="9">
         <f>G32*57.3</f>
-        <v>-1.6715597843447585</v>
+        <v>-2.3591123660993776</v>
       </c>
       <c r="H33" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:26" ht="18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:26" ht="17" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>137</v>
       </c>
@@ -10212,37 +10406,37 @@
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="21" x14ac:dyDescent="0.35">
-      <c r="H36" s="24"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="26" t="s">
+    <row r="36" spans="1:26" ht="21" x14ac:dyDescent="0.25">
+      <c r="H36" s="22"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="N36" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="O36" s="19"/>
-      <c r="P36" s="19"/>
-      <c r="Q36" s="19"/>
-      <c r="R36" s="19"/>
-      <c r="S36" s="19"/>
-      <c r="T36" s="19"/>
-      <c r="U36" s="25"/>
-      <c r="V36" s="25"/>
-      <c r="W36" s="25"/>
-      <c r="X36" s="27" t="s">
+      <c r="O36" s="17"/>
+      <c r="P36" s="17"/>
+      <c r="Q36" s="17"/>
+      <c r="R36" s="17"/>
+      <c r="S36" s="17"/>
+      <c r="T36" s="17"/>
+      <c r="U36" s="23"/>
+      <c r="V36" s="23"/>
+      <c r="W36" s="23"/>
+      <c r="X36" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="Y36" s="25"/>
-      <c r="Z36" s="25"/>
+      <c r="Y36" s="23"/>
+      <c r="Z36" s="23"/>
     </row>
-    <row r="37" spans="1:26" ht="21" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="33" t="s">
+    <row r="37" spans="1:26" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
       <c r="H37" t="s">
         <v>55</v>
       </c>
@@ -10264,7 +10458,7 @@
       <c r="N37" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="O37" s="18" t="s">
+      <c r="O37" s="16" t="s">
         <v>158</v>
       </c>
       <c r="P37" t="s">
@@ -10279,7 +10473,7 @@
       <c r="S37" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="T37" s="18" t="s">
+      <c r="T37" s="16" t="s">
         <v>159</v>
       </c>
       <c r="U37" t="s">
@@ -10291,7 +10485,7 @@
       <c r="W37" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="X37" s="18" t="s">
+      <c r="X37" s="16" t="s">
         <v>162</v>
       </c>
       <c r="Y37" s="1" t="s">
@@ -10301,7 +10495,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="38" spans="1:26" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:26" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="H38">
         <v>61</v>
       </c>
@@ -10319,19 +10513,19 @@
       </c>
       <c r="L38">
         <f>-(( (B$13 *(B$22-B$23)/(J38*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K38-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.30507856467380495</v>
-      </c>
-      <c r="M38" s="17">
+        <v>-0.31707773713025555</v>
+      </c>
+      <c r="M38" s="15">
         <f t="shared" ref="M38:M45" si="2">L38*57.3</f>
-        <v>-17.481001755809022</v>
+        <v>-18.168554337563641</v>
       </c>
       <c r="N38">
         <f>-(( (B$13 *(B$22-B$23)/(J38*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K38-Elevator!B$7)*R38)/ ((Aileron!B$11*Elevator!S38)-(R38*Elevator!B$33))</f>
-        <v>-0.34151947993960113</v>
-      </c>
-      <c r="O38" s="17">
+        <v>-0.35518355786303418</v>
+      </c>
+      <c r="O38" s="15">
         <f>N38*57.3</f>
-        <v>-19.569066200539144</v>
+        <v>-20.352017865551858</v>
       </c>
       <c r="P38">
         <f>5.2414</f>
@@ -10362,22 +10556,22 @@
       </c>
       <c r="W38">
         <f>-(( (B$13 *(B$22-B$23)/(V38*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U38-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.4258343340028577</v>
-      </c>
-      <c r="X38" s="17">
+        <v>-0.43783350645930824</v>
+      </c>
+      <c r="X38" s="15">
         <f>W38*57.3</f>
-        <v>-24.400307338363746</v>
+        <v>-25.087859920118362</v>
       </c>
       <c r="Y38">
         <f>-(( (B$13 *(B$22-B$23)/(V38*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U38-Elevator!B$7)*R38)/ ((Aileron!B$11*Elevator!S38)-(R38*Elevator!B$33))</f>
-        <v>-0.48053974672043215</v>
-      </c>
-      <c r="Z38" s="17">
+        <v>-0.4942038246438652</v>
+      </c>
+      <c r="Z38" s="15">
         <f>Y38*57.3</f>
-        <v>-27.534927487080761</v>
+        <v>-28.317879152093475</v>
       </c>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D39" t="s">
         <v>95</v>
       </c>
@@ -10405,19 +10599,19 @@
       </c>
       <c r="L39">
         <f>-(( (B$13 *(B$22-B$23)/(J39*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K39-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.26445306976647592</v>
-      </c>
-      <c r="M39" s="17">
+        <v>-0.27645224222292647</v>
+      </c>
+      <c r="M39" s="15">
         <f t="shared" si="2"/>
-        <v>-15.15316089761907</v>
+        <v>-15.840713479373687</v>
       </c>
       <c r="N39">
         <f>-(( (B$13 *(B$22-B$23)/(J39*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K39-Elevator!B$7)*R39)/ ((Aileron!B$11*Elevator!S39)-(R39*Elevator!B$33))</f>
-        <v>-0.29474931590105879</v>
-      </c>
-      <c r="O39" s="17">
+        <v>-0.30841339382449179</v>
+      </c>
+      <c r="O39" s="15">
         <f t="shared" ref="O39:O45" si="5">N39*57.3</f>
-        <v>-16.889135801130667</v>
+        <v>-17.672087466143378</v>
       </c>
       <c r="P39">
         <f t="shared" ref="P39:P45" si="6">5.2414</f>
@@ -10448,26 +10642,26 @@
       </c>
       <c r="W39">
         <f>-(( (B$13 *(B$22-B$23)/(V39*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U39-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.37080389051757767</v>
-      </c>
-      <c r="X39" s="17">
+        <v>-0.38280306297402822</v>
+      </c>
+      <c r="X39" s="15">
         <f t="shared" ref="X39:X45" si="7">W39*57.3</f>
-        <v>-21.2470629266572</v>
+        <v>-21.934615508411817</v>
       </c>
       <c r="Y39">
         <f>-(( (B$13 *(B$22-B$23)/(V39*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U39-Elevator!B$7)*R39)/ ((Aileron!B$11*Elevator!S39)-(R39*Elevator!B$33))</f>
-        <v>-0.4171858632836557</v>
-      </c>
-      <c r="Z39" s="17">
+        <v>-0.43084994120708875</v>
+      </c>
+      <c r="Z39" s="15">
         <f t="shared" ref="Z39:Z45" si="8">Y39*57.3</f>
-        <v>-23.904749966153471</v>
+        <v>-24.687701631166185</v>
       </c>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B40" s="13">
+      <c r="B40" s="12">
         <v>1</v>
       </c>
       <c r="C40" t="s">
@@ -10490,19 +10684,19 @@
       </c>
       <c r="L40">
         <f>-(( (B$13 *(B$22-B$23)/(J40*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K40-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.22313543131435182</v>
-      </c>
-      <c r="M40" s="17">
+        <v>-0.23513460377080239</v>
+      </c>
+      <c r="M40" s="15">
         <f t="shared" si="2"/>
-        <v>-12.785660214312358</v>
+        <v>-13.473212796066976</v>
       </c>
       <c r="N40">
         <f>-(( (B$13 *(B$22-B$23)/(J40*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K40-Elevator!B$7)*R40)/ ((Aileron!B$11*Elevator!S40)-(R40*Elevator!B$33))</f>
-        <v>-0.24718232053277819</v>
-      </c>
-      <c r="O40" s="17">
+        <v>-0.26084639845621116</v>
+      </c>
+      <c r="O40" s="15">
         <f t="shared" si="5"/>
-        <v>-14.163546966528189</v>
+        <v>-14.946498631540898</v>
       </c>
       <c r="P40">
         <f t="shared" si="6"/>
@@ -10533,22 +10727,22 @@
       </c>
       <c r="W40">
         <f>-(( (B$13 *(B$22-B$23)/(V40*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U40-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.31483588390076106</v>
-      </c>
-      <c r="X40" s="17">
+        <v>-0.32683505635721161</v>
+      </c>
+      <c r="X40" s="15">
         <f t="shared" si="7"/>
-        <v>-18.040096147513609</v>
+        <v>-18.727648729268225</v>
       </c>
       <c r="Y40">
         <f>-(( (B$13 *(B$22-B$23)/(V40*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U40-Elevator!B$7)*R40)/ ((Aileron!B$11*Elevator!S40)-(R40*Elevator!B$33))</f>
-        <v>-0.35275260883716025</v>
-      </c>
-      <c r="Z40" s="17">
+        <v>-0.3664166867605933</v>
+      </c>
+      <c r="Z40" s="15">
         <f t="shared" si="8"/>
-        <v>-20.212724486369282</v>
+        <v>-20.995676151381996</v>
       </c>
     </row>
-    <row r="41" spans="1:26" ht="18" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:26" ht="17" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>100</v>
       </c>
@@ -10562,7 +10756,7 @@
       <c r="D41" t="s">
         <v>97</v>
       </c>
-      <c r="E41" s="28">
+      <c r="E41" s="26">
         <f>B29*B42</f>
         <v>0.45219275698941064</v>
       </c>
@@ -10586,19 +10780,19 @@
       </c>
       <c r="L41">
         <f>-(( (B$13 *(B$22-B$23)/(J41*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K41-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.16252188184899624</v>
-      </c>
-      <c r="M41" s="17">
+        <v>-0.17452105430544687</v>
+      </c>
+      <c r="M41" s="15">
         <f t="shared" si="2"/>
-        <v>-9.3125038299474845</v>
+        <v>-10.000056411702106</v>
       </c>
       <c r="N41">
         <f>-(( (B$13 *(B$22-B$23)/(J41*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K41-Elevator!B$7)*R41)/ ((Aileron!B$11*Elevator!S41)-(R41*Elevator!B$33))</f>
-        <v>-0.17740087767479715</v>
-      </c>
-      <c r="O41" s="17">
+        <v>-0.19106495559823017</v>
+      </c>
+      <c r="O41" s="15">
         <f t="shared" si="5"/>
-        <v>-10.165070290765875</v>
+        <v>-10.948021955778588</v>
       </c>
       <c r="P41">
         <f t="shared" si="6"/>
@@ -10629,22 +10823,22 @@
       </c>
       <c r="W41">
         <f>-(( (B$13 *(B$22-B$23)/(V41*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U41-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.23273004086046584</v>
-      </c>
-      <c r="X41" s="17">
+        <v>-0.24472921331691641</v>
+      </c>
+      <c r="X41" s="15">
         <f t="shared" si="7"/>
-        <v>-13.335431341304691</v>
+        <v>-14.022983923059309</v>
       </c>
       <c r="Y41">
         <f>-(( (B$13 *(B$22-B$23)/(V41*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U41-Elevator!B$7)*R41)/ ((Aileron!B$11*Elevator!S41)-(R41*Elevator!B$33))</f>
-        <v>-0.25822812965783976</v>
-      </c>
-      <c r="Z41" s="17">
+        <v>-0.27189220758127269</v>
+      </c>
+      <c r="Z41" s="15">
         <f t="shared" si="8"/>
-        <v>-14.796471829394218</v>
+        <v>-15.579423494406925</v>
       </c>
     </row>
-    <row r="42" spans="1:26" ht="18" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:26" ht="17" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>99</v>
       </c>
@@ -10652,7 +10846,6 @@
         <f>Aileron!B8/Elevator!E39</f>
         <v>1.2919793056840305</v>
       </c>
-      <c r="E42" s="16"/>
       <c r="H42">
         <v>100</v>
       </c>
@@ -10670,19 +10863,19 @@
       </c>
       <c r="L42">
         <f>-(( (B$13 *(B$22-B$23)/(J42*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K42-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-9.1240347677738115E-2</v>
-      </c>
-      <c r="M42" s="17">
+        <v>-0.1032395201341887</v>
+      </c>
+      <c r="M42" s="15">
         <f t="shared" si="2"/>
-        <v>-5.2280719219343936</v>
+        <v>-5.9156245036890125</v>
       </c>
       <c r="N42">
         <f>-(( (B$13 *(B$22-B$23)/(J42*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K42-Elevator!B$7)*R42)/ ((Aileron!B$11*Elevator!S42)-(R42*Elevator!B$33))</f>
-        <v>-9.5337900873811485E-2</v>
-      </c>
-      <c r="O42" s="17">
+        <v>-0.10900197879724448</v>
+      </c>
+      <c r="O42" s="15">
         <f t="shared" si="5"/>
-        <v>-5.4628617200693981</v>
+        <v>-6.2458133850821085</v>
       </c>
       <c r="P42">
         <f t="shared" si="6"/>
@@ -10713,26 +10906,26 @@
       </c>
       <c r="W42">
         <f>-(( (B$13 *(B$22-B$23)/(V42*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U42-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-0.13617356944507861</v>
-      </c>
-      <c r="X42" s="17">
+        <v>-0.14817274190152921</v>
+      </c>
+      <c r="X42" s="15">
         <f t="shared" si="7"/>
-        <v>-7.8027455292030039</v>
+        <v>-8.4902981109576228</v>
       </c>
       <c r="Y42">
         <f>-(( (B$13 *(B$22-B$23)/(V42*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U42-Elevator!B$7)*R42)/ ((Aileron!B$11*Elevator!S42)-(R42*Elevator!B$33))</f>
-        <v>-0.14706734214295869</v>
-      </c>
-      <c r="Z42" s="17">
+        <v>-0.16073142006639171</v>
+      </c>
+      <c r="Z42" s="15">
         <f t="shared" si="8"/>
-        <v>-8.4269587047915326</v>
+        <v>-9.2099103698042448</v>
       </c>
     </row>
-    <row r="43" spans="1:26" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:26" ht="18" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B43" s="28">
+      <c r="B43" s="26">
         <f>B41*E41</f>
         <v>2.2200499999999996</v>
       </c>
@@ -10756,19 +10949,19 @@
       </c>
       <c r="L43">
         <f>-(( (B$13 *(B$22-B$23)/(J43*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K43-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-5.2519514300758338E-2</v>
-      </c>
-      <c r="M43" s="17">
+        <v>-6.451868675720894E-2</v>
+      </c>
+      <c r="M43" s="15">
         <f t="shared" si="2"/>
-        <v>-3.0093681694334524</v>
+        <v>-3.6969207511880722</v>
       </c>
       <c r="N43">
         <f>-(( (B$13 *(B$22-B$23)/(J43*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K43-Elevator!B$7)*R43)/ ((Aileron!B$11*Elevator!S43)-(R43*Elevator!B$33))</f>
-        <v>-5.0760481376979714E-2</v>
-      </c>
-      <c r="O43" s="17">
+        <v>-6.4424559300412729E-2</v>
+      </c>
+      <c r="O43" s="15">
         <f t="shared" si="5"/>
-        <v>-2.9085755829009377</v>
+        <v>-3.6915272479136494</v>
       </c>
       <c r="P43">
         <f t="shared" si="6"/>
@@ -10799,22 +10992,22 @@
       </c>
       <c r="W43">
         <f>-(( (B$13 *(B$22-B$23)/(V43*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U43-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-8.3723140528078152E-2</v>
-      </c>
-      <c r="X43" s="17">
+        <v>-9.572231298452874E-2</v>
+      </c>
+      <c r="X43" s="15">
         <f t="shared" si="7"/>
-        <v>-4.7973359522588774</v>
+        <v>-5.4848885340134963</v>
       </c>
       <c r="Y43">
         <f>-(( (B$13 *(B$22-B$23)/(V43*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U43-Elevator!B$7)*R43)/ ((Aileron!B$11*Elevator!S43)-(R43*Elevator!B$33))</f>
-        <v>-8.6683704480554194E-2</v>
-      </c>
-      <c r="Z43" s="17">
+        <v>-0.10034778240398719</v>
+      </c>
+      <c r="Z43" s="15">
         <f t="shared" si="8"/>
-        <v>-4.9669762667357551</v>
+        <v>-5.7499279317484655</v>
       </c>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.2">
       <c r="H44">
         <v>140</v>
       </c>
@@ -10832,19 +11025,19 @@
       </c>
       <c r="L44">
         <f>-(( (B$13 *(B$22-B$23)/(J44*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K44-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-2.9172073025213938E-2</v>
-      </c>
-      <c r="M44" s="17">
+        <v>-4.117124548166453E-2</v>
+      </c>
+      <c r="M44" s="15">
         <f t="shared" si="2"/>
-        <v>-1.6715597843447585</v>
+        <v>-2.3591123660993776</v>
       </c>
       <c r="N44">
         <f>-(( (B$13 *(B$22-B$23)/(J44*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K44-Elevator!B$7)*R44)/ ((Aileron!B$11*Elevator!S44)-(R44*Elevator!B$33))</f>
-        <v>-2.3881703387238832E-2</v>
-      </c>
-      <c r="O44" s="17">
+        <v>-3.7545781310671836E-2</v>
+      </c>
+      <c r="O44" s="15">
         <f t="shared" si="5"/>
-        <v>-1.3684216040887851</v>
+        <v>-2.1513732691014962</v>
       </c>
       <c r="P44">
         <f t="shared" si="6"/>
@@ -10875,22 +11068,22 @@
       </c>
       <c r="W44">
         <f>-(( (B$13 *(B$22-B$23)/(V44*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U44-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-5.2097186171816239E-2</v>
-      </c>
-      <c r="X44" s="17">
+        <v>-6.4096358628266834E-2</v>
+      </c>
+      <c r="X44" s="15">
         <f t="shared" si="7"/>
-        <v>-2.9851687676450704</v>
+        <v>-3.6727213493996893</v>
       </c>
       <c r="Y44">
         <f>-(( (B$13 *(B$22-B$23)/(V44*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U44-Elevator!B$7)*R44)/ ((Aileron!B$11*Elevator!S44)-(R44*Elevator!B$33))</f>
-        <v>-5.0274275463334357E-2</v>
-      </c>
-      <c r="Z44" s="17">
+        <v>-6.3938353386767358E-2</v>
+      </c>
+      <c r="Z44" s="15">
         <f t="shared" si="8"/>
-        <v>-2.8807159840490586</v>
+        <v>-3.6636676490617694</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.2">
       <c r="H45">
         <v>170</v>
       </c>
@@ -10908,19 +11101,19 @@
       </c>
       <c r="L45">
         <f>-(( (B$13 *(B$22-B$23)/(J45*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K45-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-8.3663148696317031E-3</v>
-      </c>
-      <c r="M45" s="17">
+        <v>-2.0365487326082295E-2</v>
+      </c>
+      <c r="M45" s="15">
         <f t="shared" si="2"/>
-        <v>-0.47938984202989654</v>
+        <v>-1.1669424237845154</v>
       </c>
       <c r="N45">
         <f>-(( (B$13 *(B$22-B$23)/(J45*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(Elevator!K45-Elevator!B$7)*R45)/ ((Aileron!B$11*Elevator!S45)-(R45*Elevator!B$33))</f>
-        <v>7.0957967472967155E-5</v>
-      </c>
-      <c r="O45" s="17">
+        <v>-1.3593119955960032E-2</v>
+      </c>
+      <c r="O45" s="15">
         <f t="shared" si="5"/>
-        <v>4.0658915362010179E-3</v>
+        <v>-0.77888577347650978</v>
       </c>
       <c r="P45">
         <f t="shared" si="6"/>
@@ -10951,19 +11144,19 @@
       </c>
       <c r="W45">
         <f>-(( (B$13 *(B$22-B$23)/(V45*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U45-Elevator!B$7)*Elevator!G$29)/ ((Aileron!B$11*Elevator!B$32)-(Elevator!G$29*Elevator!B$33))</f>
-        <v>-2.3914142470787589E-2</v>
-      </c>
-      <c r="X45" s="17">
+        <v>-3.5913314927238184E-2</v>
+      </c>
+      <c r="X45" s="15">
         <f t="shared" si="7"/>
-        <v>-1.3702803635761287</v>
+        <v>-2.0578329453307478</v>
       </c>
       <c r="Y45">
         <f>-(( (B$13 *(B$22-B$23)/(V45*Aileron!B$7*Aileron!B$15)+E$8))*Aileron!B$11 +(U45-Elevator!B$7)*R45)/ ((Aileron!B$11*Elevator!S45)-(R45*Elevator!B$33))</f>
-        <v>-1.7828502679290776E-2</v>
-      </c>
-      <c r="Z45" s="17">
+        <v>-3.149258060272378E-2</v>
+      </c>
+      <c r="Z45" s="15">
         <f t="shared" si="8"/>
-        <v>-1.0215732035233613</v>
+        <v>-1.8045248685360724</v>
       </c>
     </row>
   </sheetData>
@@ -10987,19 +11180,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A2:O40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="9.7109375" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" ht="18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="10">
         <v>3.9496000000000002</v>
       </c>
       <c r="C2" t="s">
@@ -11008,7 +11201,7 @@
       <c r="D2" t="s">
         <v>163</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="10">
         <v>20</v>
       </c>
       <c r="F2" t="s">
@@ -11024,25 +11217,25 @@
       <c r="I2" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="34" t="s">
+      <c r="K2" s="31" t="s">
         <v>213</v>
       </c>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
     </row>
-    <row r="3" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3">
         <f>SQRT(B2*K3)</f>
         <v>2.3514761321348767</v>
       </c>
       <c r="D3" t="s">
         <v>167</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="17">
         <f>4.6-(0.17*1.7684)</f>
         <v>4.299372</v>
       </c>
@@ -11052,7 +11245,7 @@
       <c r="G3" t="s">
         <v>124</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <v>4.122522</v>
       </c>
       <c r="I3" t="s">
@@ -11067,18 +11260,18 @@
       <c r="M3" t="s">
         <v>212</v>
       </c>
-      <c r="N3" s="11">
+      <c r="N3" s="10">
         <v>0.10100000000000001</v>
       </c>
       <c r="O3" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>101</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4">
         <f>N4/(1+(N4/(3.142*K3)))</f>
         <v>2.4992072765827937</v>
       </c>
@@ -11115,11 +11308,11 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <v>0.97</v>
       </c>
       <c r="D5" t="s">
@@ -11139,11 +11332,11 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="10">
         <v>0</v>
       </c>
       <c r="J6" t="s">
@@ -11154,11 +11347,11 @@
         <v>1.6796258086677691</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <v>0</v>
       </c>
       <c r="D7" t="s">
@@ -11179,11 +11372,11 @@
         <v>1.8118412513325792</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <v>0</v>
       </c>
       <c r="C8" t="s">
@@ -11192,7 +11385,7 @@
       <c r="D8" t="s">
         <v>114</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="17">
         <f>E7-(2.6+0.4*1.7684)</f>
         <v>2.3148712025699796</v>
       </c>
@@ -11206,11 +11399,11 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="18.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" ht="18" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <v>9.7170000000000005</v>
       </c>
       <c r="C9" t="s">
@@ -11227,7 +11420,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>108</v>
       </c>
@@ -11242,7 +11435,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>110</v>
       </c>
@@ -11256,18 +11449,18 @@
       <c r="D11" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="10">
         <v>1</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="10">
         <f>0.3</f>
         <v>0.3</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>112</v>
       </c>
@@ -11281,17 +11474,17 @@
       <c r="D12" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="10">
         <v>0.51</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>113</v>
       </c>
@@ -11313,11 +11506,11 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <f>B2*E3/(Aileron!B13*Aileron!B7)</f>
         <v>5.1870507334625074E-2</v>
       </c>
@@ -11332,21 +11525,21 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="D15" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="10">
         <v>0.75</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="10">
         <v>1.35</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>120</v>
       </c>
@@ -11368,7 +11561,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>121</v>
       </c>
@@ -11390,30 +11583,30 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A19" s="17" t="s">
+    <row r="19" spans="1:13" ht="17" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="18" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F20)/Rudder!B$16)</f>
         <v>2.2766641797327685</v>
@@ -11434,7 +11627,7 @@
         <f t="shared" ref="E20:E26" si="1">D20+(E$9*E$8*COS(F20))</f>
         <v>-17110.094281583057</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="10">
         <v>-0.5</v>
       </c>
       <c r="G20">
@@ -11442,7 +11635,7 @@
         <v>-28.65</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F21)/Rudder!B$16)</f>
         <v>1.4825465326739451</v>
@@ -11463,7 +11656,7 @@
         <f t="shared" si="1"/>
         <v>-11060.615577844104</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="10">
         <v>-0.2</v>
       </c>
       <c r="G21">
@@ -11471,7 +11664,7 @@
         <v>-11.46</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F22)/Rudder!B$16)</f>
         <v>1.217840650321004</v>
@@ -11492,7 +11685,7 @@
         <f t="shared" si="1"/>
         <v>-9076.2450727825144</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="10">
         <v>-0.1</v>
       </c>
       <c r="G22">
@@ -11500,7 +11693,7 @@
         <v>-5.73</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F23)/Rudder!B$16)</f>
         <v>0.95313476796806262</v>
@@ -11521,7 +11714,7 @@
         <f t="shared" si="1"/>
         <v>-7108.4869820165968</v>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="10">
         <v>0</v>
       </c>
       <c r="G23">
@@ -11529,7 +11722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F24)/Rudder!B$16)</f>
         <v>2.6664179732768467E-2</v>
@@ -11550,7 +11743,7 @@
         <f t="shared" si="1"/>
         <v>-351.85800099623589</v>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="10">
         <v>0.35</v>
       </c>
       <c r="G24">
@@ -11558,7 +11751,7 @@
         <v>20.054999999999996</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F25)/Rudder!B$16)</f>
         <v>-9.7064085025257985E-3</v>
@@ -11579,7 +11772,7 @@
         <f t="shared" si="1"/>
         <v>-90.655614613250009</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="10">
         <v>0.36374000000000001</v>
       </c>
       <c r="G25">
@@ -11587,7 +11780,7 @@
         <v>20.842302</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26">
         <f>(E$9/(0.5*1.225*E$5^2*Aileron!B$7*Rudder!B$16))-((Rudder!E$17*Rudder!E$13)/Rudder!B$16)+((Rudder!E$17*Rudder!F26)/Rudder!B$16)</f>
         <v>-2.0982879090761131E-2</v>
@@ -11608,7 +11801,7 @@
         <f t="shared" si="1"/>
         <v>-9.7314134532366552</v>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="10">
         <v>0.36799999999999999</v>
       </c>
       <c r="G26">
@@ -11616,49 +11809,47 @@
         <v>21.086399999999998</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="C28" s="21" t="s">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C28" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="17"/>
     </row>
-    <row r="29" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="C29" s="21" t="s">
+    <row r="29" spans="1:13" ht="17" x14ac:dyDescent="0.25">
+      <c r="C29" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
     </row>
-    <row r="31" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" ht="17" x14ac:dyDescent="0.25">
       <c r="G31" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="10">
         <v>0.36799999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A32" s="36" t="s">
+    <row r="32" spans="1:13" ht="17" x14ac:dyDescent="0.25">
+      <c r="A32" s="33" t="s">
         <v>174</v>
       </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
       <c r="G32" s="4" t="s">
         <v>77</v>
       </c>
@@ -11666,14 +11857,14 @@
         <f>H31*57.3</f>
         <v>21.086399999999998</v>
       </c>
-      <c r="J32" s="23" t="s">
+      <c r="J32" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17"/>
+      <c r="M32" s="17"/>
     </row>
-    <row r="33" spans="1:14" ht="18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>125</v>
       </c>
@@ -11690,14 +11881,14 @@
       <c r="H33">
         <v>30</v>
       </c>
-      <c r="K33" s="21" t="s">
+      <c r="K33" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="L33" s="19"/>
-      <c r="M33" s="19"/>
-      <c r="N33" s="19"/>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+      <c r="N33" s="17"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B34" s="4" t="s">
         <v>77</v>
       </c>
@@ -11708,12 +11899,12 @@
       <c r="D34" t="s">
         <v>24</v>
       </c>
-      <c r="K34" s="21" t="s">
+      <c r="K34" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="L34" s="19"/>
+      <c r="L34" s="17"/>
     </row>
-    <row r="35" spans="1:14" ht="18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" ht="17" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>126</v>
       </c>
@@ -11724,8 +11915,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="E36" s="17" t="s">
+    <row r="36" spans="1:14" ht="17" x14ac:dyDescent="0.25">
+      <c r="E36" s="15" t="s">
         <v>133</v>
       </c>
       <c r="F36">
@@ -11736,15 +11927,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="35" t="s">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A37" s="32" t="s">
         <v>128</v>
       </c>
-      <c r="B37" s="35"/>
+      <c r="B37" s="32"/>
       <c r="E37" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F37" s="28">
+      <c r="F37" s="26">
         <f>F36/0.514</f>
         <v>43.235967371918832</v>
       </c>
@@ -11752,11 +11943,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>129</v>
       </c>
-      <c r="B38" s="28">
+      <c r="B38" s="26">
         <f>G11*B11</f>
         <v>0.50388774260033076</v>
       </c>
@@ -11764,11 +11955,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>130</v>
       </c>
-      <c r="B39" s="28">
+      <c r="B39" s="26">
         <f>E11*B3</f>
         <v>2.3514761321348767</v>
       </c>
@@ -11776,11 +11967,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="17.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>132</v>
       </c>
-      <c r="B40" s="28">
+      <c r="B40" s="26">
         <f>B38*B39</f>
         <v>1.1848800000000002</v>
       </c>

</xml_diff>